<commit_message>
Fix radiotherapy CRF typos in CRF_PR_RS workbook
- THERAPHY -> THERAPY in PRCAT prepopulated terms (prior and subsequent)
- SUBSEQUENTRADTHERAPY PRCAT annotation now says SUBSEQUENT, not PRIOR
- cGY -> cGy in the dose-unit value lists (matches CDISC UNIT terminology)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/curation/draft/crf/CRF_PR_RS_RadioTherapy.xlsx
+++ b/curation/draft/crf/CRF_PR_RS_RadioTherapy.xlsx
@@ -114,7 +114,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="985" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="985" uniqueCount="241">
   <si>
     <t>This spreadsheet contains CDISC CRF Specializations loaded from 303 YAML files as of 2025-11-26.
 The spreadsheet contains 303 unique CDISC CRF Specializations.
@@ -457,7 +457,7 @@
     <t>Procedure Category</t>
   </si>
   <si>
-    <t>PRIOR RADIATION THERAPHY</t>
+    <t>PRIOR RADIATION THERAPY</t>
   </si>
   <si>
     <t>PRCAT = PRIOR RADIATION THERAPY</t>
@@ -643,7 +643,7 @@
     <t>UNIT</t>
   </si>
   <si>
-    <t>Gy;Rad;cGY</t>
+    <t>Gy;Rad;cGy</t>
   </si>
   <si>
     <t>PRDOSU</t>
@@ -781,7 +781,7 @@
     <t>3D CONFORMAL RADIATION THERAPY;INTENSITY-MODULATED RADIATION THERAPY;RADIOSURGERY;STEREOTACTIC BODY RADIATION THERAPY;TOTAL BODY IRRADIATION;BRACHYTHERAPY, INTRACAVITARY;BRACHYTHERAPY, INTERSTITIAL;RADIOEMBOLIZATION</t>
   </si>
   <si>
-    <t>SUBSEQUENT RADIATION THERAPHY</t>
+    <t>SUBSEQUENT RADIATION THERAPY</t>
   </si>
   <si>
     <t>Was Subsequent Radiotherapy Performed?</t>
@@ -876,6 +876,9 @@
   </si>
   <si>
     <t>PRTRTSTT in SUPPPR; if NOT APPLICABLE is selected then NOT SUBMITTED</t>
+  </si>
+  <si>
+    <t>PRCAT = SUBSEQUENT RADIATION THERAPY</t>
   </si>
 </sst>
 </file>
@@ -4153,7 +4156,7 @@
         <v>110</v>
       </c>
       <c r="AI29" s="18" t="s">
-        <v>114</v>
+        <v>240</v>
       </c>
     </row>
     <row r="30" spans="1:35" ht="12" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>